<commit_message>
Add game data: Friendly fire, Ich vermisse schlechte Laune nach unnötigen Chatnachrichten
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2394,7 +2394,84 @@
       <c r="H49" t="n">
         <v>1</v>
       </c>
+      <c r="I49" t="n">
+        <v/>
+      </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>6a9d3570da7652b981a8ac1c</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Friendly fire</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>10</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F50" t="n">
+        <v>5</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>6a8c93f4caed5916708ea5e4</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ich vermisse schlechte Laune nach unnötigen Chatnachrichten</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2411,7 +2488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6213,6 +6290,144 @@
         </is>
       </c>
       <c r="E165" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>6a9d3570da7652b981a8ac1c</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>10</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Winnu</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6a9d3570da7652b981a8ac1c</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>4</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Muaat</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>6a9d3570da7652b981a8ac1c</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>4</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Sardakk</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>6a8c93f4caed5916708ea5e4</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>8</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>6a8c93f4caed5916708ea5e4</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>10</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Arborec</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>6a8c93f4caed5916708ea5e4</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>8</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Yin</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: Dude, where is my skip?
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2434,6 +2434,9 @@
       <c r="H50" t="n">
         <v>1</v>
       </c>
+      <c r="I50" t="n">
+        <v/>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>online</t>
@@ -2471,7 +2474,47 @@
       <c r="H51" t="n">
         <v>1</v>
       </c>
+      <c r="I51" t="n">
+        <v/>
+      </c>
       <c r="J51" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>6aa276baf2fff42429b2341d</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Dude, where is my skip?</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="F52" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2488,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E174"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6428,6 +6471,75 @@
         </is>
       </c>
       <c r="E171" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>6aa276baf2fff42429b2341d</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>10</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Mentak</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>6aa276baf2fff42429b2341d</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>5</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>The L1Z1X Mindnet</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>6aa276baf2fff42429b2341d</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>8</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Naalu</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: Skippedyskip
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2514,7 +2514,47 @@
       <c r="H52" t="n">
         <v>1</v>
       </c>
+      <c r="I52" t="n">
+        <v/>
+      </c>
       <c r="J52" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>6ab28f6cc72eb32447571861</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Skippedyskip</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>10</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F53" t="n">
+        <v>6</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2531,7 +2571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6540,6 +6580,75 @@
         </is>
       </c>
       <c r="E174" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>6ab28f6cc72eb32447571861</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>9</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Xxcha</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>6ab28f6cc72eb32447571861</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>7</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Sardakk</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>6ab28f6cc72eb32447571861</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>10</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Hacan</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge duplicate L1Z1X faction entry (The L1Z1X Mindnet → L1Z1X)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S8Z7iW9Sdu9k9cdWRbBN5R
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -523,9 +523,6 @@
           <t>Statusphase, Starki Naalu 3 VP mit Public und Sekret</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -563,9 +560,6 @@
           <t xml:space="preserve">Statusphase, Manu Jol 2 VP mit 1 Public und Sekret, hatte auch Imperial aber nur für 1 PO (nicht MR) in Runde. Speaker letzte Runde war Eric </t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,9 +597,6 @@
           <t>Aktionsphase: Manu spielt Imperial und scort Lead from the Front</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -643,9 +634,6 @@
           <t>Eric in Aktionphase, hatte auch Imperial für 2 VP PO, Sieg aber unklar warum</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -683,9 +671,6 @@
           <t>Win in Agendaphase, da Political Censure</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -723,9 +708,6 @@
           <t>Sieg Eric in Aktionphase durch Sekret Destroy Their greatest ship</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -763,9 +745,6 @@
           <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -803,9 +782,6 @@
           <t>Thomas in Statusphase 2 VP mit PO</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -843,9 +819,6 @@
           <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -883,9 +856,6 @@
           <t>Eric in Statusphase mit 2VP PO</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -923,9 +893,6 @@
           <t>Eric in Agendaphase mit Crown of Emphidia</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -963,9 +930,6 @@
           <t>Frank, Aktionsphase, Sekret Destroy their greatest Ship</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1003,9 +967,6 @@
           <t>Manu, Aktionsphase, Sekret Destroy their greatest Ship</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1043,9 +1004,6 @@
           <t>Eric, Statusphase 1 VP mit Sekret</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1083,9 +1041,6 @@
           <t>Frank, Statusphase 1 VP mit PO</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1123,9 +1078,6 @@
           <t>Thomas, Statusphase, 1 VP mit PO</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1163,9 +1115,6 @@
           <t>Thomas durch Support Trade</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1203,9 +1152,6 @@
           <t>Manu in Statusphase, 2 VP mit PO</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1243,9 +1189,6 @@
           <t>Eric in Aktionsphase mit Imperial, 1 VP PO und 1 VP MR</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1283,9 +1226,6 @@
           <t>Thomas in Statusphase 1 VP mit PO</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1323,9 +1263,6 @@
           <t>Manu in Statusphase, 1 VP mit PO</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1363,9 +1300,6 @@
           <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1403,9 +1337,6 @@
           <t>Thomas in Aktionsphase mit Sekret Destroy Their greates Ship</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1443,9 +1374,6 @@
           <t>Eric in Aktionsphase durch Shard of the Throne</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1483,9 +1411,6 @@
           <t>Eric in Agendaphase durch Mutiny</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1523,9 +1448,6 @@
           <t>Manu in Aktionsphase durch Spark a Rebellion</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1563,9 +1485,6 @@
           <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1603,9 +1522,6 @@
           <t>Thomas in Statusphase 2 VP durch PO</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1643,9 +1559,6 @@
           <t>Eric in Statusphase mit 3VP, 2 PO und 1 Sekret</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1683,9 +1596,6 @@
           <t>Eric in Aktionsphase, Demonstrate your Power</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1723,9 +1633,6 @@
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1763,9 +1670,6 @@
           <t>Manu in Statusphase, 1 VP mit PO</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1803,9 +1707,6 @@
           <t>Thomas in Aktionsphase mit Imperial und 2 VP PO</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1843,9 +1744,6 @@
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1883,9 +1781,6 @@
           <t>Thomas in Aktionsphase 1 VP mit Imperial MR</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1923,9 +1818,6 @@
           <t>Manu in Aktionsphase 2 VP mit Imperial PO</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1963,9 +1855,6 @@
           <t>Frank in Statusphase 2 VP.</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v/>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2003,9 +1892,6 @@
           <t>Eric hatte 9 Punkte; Shard of Throne gefunden. Damit war spiel fertig.</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2038,12 +1924,6 @@
       <c r="H40" t="n">
         <v>0</v>
       </c>
-      <c r="I40" t="n">
-        <v/>
-      </c>
-      <c r="J40" t="n">
-        <v/>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2081,9 +1961,6 @@
           <t>Manu hatte imperial und ein noch ein offenes 1er PO</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v/>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2116,12 +1993,6 @@
       <c r="H42" t="n">
         <v>0</v>
       </c>
-      <c r="I42" t="n">
-        <v/>
-      </c>
-      <c r="J42" t="n">
-        <v/>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2154,9 +2025,6 @@
       <c r="H43" t="n">
         <v>1</v>
       </c>
-      <c r="I43" t="n">
-        <v/>
-      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>online</t>
@@ -2194,9 +2062,6 @@
       <c r="H44" t="n">
         <v>1</v>
       </c>
-      <c r="I44" t="n">
-        <v/>
-      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>online</t>
@@ -2234,9 +2099,6 @@
       <c r="H45" t="n">
         <v>1</v>
       </c>
-      <c r="I45" t="n">
-        <v/>
-      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>online</t>
@@ -2274,9 +2136,6 @@
       <c r="H46" t="n">
         <v>1</v>
       </c>
-      <c r="I46" t="n">
-        <v/>
-      </c>
       <c r="J46" t="inlineStr">
         <is>
           <t>online</t>
@@ -2314,9 +2173,6 @@
       <c r="H47" t="n">
         <v>1</v>
       </c>
-      <c r="I47" t="n">
-        <v/>
-      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>online</t>
@@ -2354,9 +2210,6 @@
       <c r="H48" t="n">
         <v>1</v>
       </c>
-      <c r="I48" t="n">
-        <v/>
-      </c>
       <c r="J48" t="inlineStr">
         <is>
           <t>online</t>
@@ -2394,9 +2247,6 @@
       <c r="H49" t="n">
         <v>1</v>
       </c>
-      <c r="I49" t="n">
-        <v/>
-      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>online</t>
@@ -2434,9 +2284,6 @@
       <c r="H50" t="n">
         <v>1</v>
       </c>
-      <c r="I50" t="n">
-        <v/>
-      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>online</t>
@@ -2474,9 +2321,6 @@
       <c r="H51" t="n">
         <v>1</v>
       </c>
-      <c r="I51" t="n">
-        <v/>
-      </c>
       <c r="J51" t="inlineStr">
         <is>
           <t>online</t>
@@ -2513,9 +2357,6 @@
       </c>
       <c r="H52" t="n">
         <v>1</v>
-      </c>
-      <c r="I52" t="n">
-        <v/>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -6553,7 +6394,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>The L1Z1X Mindnet</t>
+          <t>L1Z1X</t>
         </is>
       </c>
       <c r="E173" t="n">

</xml_diff>

<commit_message>
Add game data: Dumm, des isses!
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -523,6 +523,9 @@
           <t>Statusphase, Starki Naalu 3 VP mit Public und Sekret</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,6 +563,9 @@
           <t xml:space="preserve">Statusphase, Manu Jol 2 VP mit 1 Public und Sekret, hatte auch Imperial aber nur für 1 PO (nicht MR) in Runde. Speaker letzte Runde war Eric </t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -597,6 +603,9 @@
           <t>Aktionsphase: Manu spielt Imperial und scort Lead from the Front</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -634,6 +643,9 @@
           <t>Eric in Aktionphase, hatte auch Imperial für 2 VP PO, Sieg aber unklar warum</t>
         </is>
       </c>
+      <c r="J5" t="n">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -671,6 +683,9 @@
           <t>Win in Agendaphase, da Political Censure</t>
         </is>
       </c>
+      <c r="J6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -708,6 +723,9 @@
           <t>Sieg Eric in Aktionphase durch Sekret Destroy Their greatest ship</t>
         </is>
       </c>
+      <c r="J7" t="n">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -745,6 +763,9 @@
           <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
         </is>
       </c>
+      <c r="J8" t="n">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -782,6 +803,9 @@
           <t>Thomas in Statusphase 2 VP mit PO</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -819,6 +843,9 @@
           <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
         </is>
       </c>
+      <c r="J10" t="n">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -856,6 +883,9 @@
           <t>Eric in Statusphase mit 2VP PO</t>
         </is>
       </c>
+      <c r="J11" t="n">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -893,6 +923,9 @@
           <t>Eric in Agendaphase mit Crown of Emphidia</t>
         </is>
       </c>
+      <c r="J12" t="n">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -930,6 +963,9 @@
           <t>Frank, Aktionsphase, Sekret Destroy their greatest Ship</t>
         </is>
       </c>
+      <c r="J13" t="n">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -967,6 +1003,9 @@
           <t>Manu, Aktionsphase, Sekret Destroy their greatest Ship</t>
         </is>
       </c>
+      <c r="J14" t="n">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1004,6 +1043,9 @@
           <t>Eric, Statusphase 1 VP mit Sekret</t>
         </is>
       </c>
+      <c r="J15" t="n">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1041,6 +1083,9 @@
           <t>Frank, Statusphase 1 VP mit PO</t>
         </is>
       </c>
+      <c r="J16" t="n">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1078,6 +1123,9 @@
           <t>Thomas, Statusphase, 1 VP mit PO</t>
         </is>
       </c>
+      <c r="J17" t="n">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1115,6 +1163,9 @@
           <t>Thomas durch Support Trade</t>
         </is>
       </c>
+      <c r="J18" t="n">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1152,6 +1203,9 @@
           <t>Manu in Statusphase, 2 VP mit PO</t>
         </is>
       </c>
+      <c r="J19" t="n">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1189,6 +1243,9 @@
           <t>Eric in Aktionsphase mit Imperial, 1 VP PO und 1 VP MR</t>
         </is>
       </c>
+      <c r="J20" t="n">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1226,6 +1283,9 @@
           <t>Thomas in Statusphase 1 VP mit PO</t>
         </is>
       </c>
+      <c r="J21" t="n">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1263,6 +1323,9 @@
           <t>Manu in Statusphase, 1 VP mit PO</t>
         </is>
       </c>
+      <c r="J22" t="n">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1300,6 +1363,9 @@
           <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
         </is>
       </c>
+      <c r="J23" t="n">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1337,6 +1403,9 @@
           <t>Thomas in Aktionsphase mit Sekret Destroy Their greates Ship</t>
         </is>
       </c>
+      <c r="J24" t="n">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1374,6 +1443,9 @@
           <t>Eric in Aktionsphase durch Shard of the Throne</t>
         </is>
       </c>
+      <c r="J25" t="n">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1411,6 +1483,9 @@
           <t>Eric in Agendaphase durch Mutiny</t>
         </is>
       </c>
+      <c r="J26" t="n">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1448,6 +1523,9 @@
           <t>Manu in Aktionsphase durch Spark a Rebellion</t>
         </is>
       </c>
+      <c r="J27" t="n">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1485,6 +1563,9 @@
           <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
         </is>
       </c>
+      <c r="J28" t="n">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1522,6 +1603,9 @@
           <t>Thomas in Statusphase 2 VP durch PO</t>
         </is>
       </c>
+      <c r="J29" t="n">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1559,6 +1643,9 @@
           <t>Eric in Statusphase mit 3VP, 2 PO und 1 Sekret</t>
         </is>
       </c>
+      <c r="J30" t="n">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1596,6 +1683,9 @@
           <t>Eric in Aktionsphase, Demonstrate your Power</t>
         </is>
       </c>
+      <c r="J31" t="n">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1633,6 +1723,9 @@
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
         </is>
       </c>
+      <c r="J32" t="n">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1670,6 +1763,9 @@
           <t>Manu in Statusphase, 1 VP mit PO</t>
         </is>
       </c>
+      <c r="J33" t="n">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1707,6 +1803,9 @@
           <t>Thomas in Aktionsphase mit Imperial und 2 VP PO</t>
         </is>
       </c>
+      <c r="J34" t="n">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1744,6 +1843,9 @@
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
         </is>
       </c>
+      <c r="J35" t="n">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1781,6 +1883,9 @@
           <t>Thomas in Aktionsphase 1 VP mit Imperial MR</t>
         </is>
       </c>
+      <c r="J36" t="n">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1818,6 +1923,9 @@
           <t>Manu in Aktionsphase 2 VP mit Imperial PO</t>
         </is>
       </c>
+      <c r="J37" t="n">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1855,6 +1963,9 @@
           <t>Frank in Statusphase 2 VP.</t>
         </is>
       </c>
+      <c r="J38" t="n">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1892,6 +2003,9 @@
           <t>Eric hatte 9 Punkte; Shard of Throne gefunden. Damit war spiel fertig.</t>
         </is>
       </c>
+      <c r="J39" t="n">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1924,6 +2038,12 @@
       <c r="H40" t="n">
         <v>0</v>
       </c>
+      <c r="I40" t="n">
+        <v/>
+      </c>
+      <c r="J40" t="n">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1961,6 +2081,9 @@
           <t>Manu hatte imperial und ein noch ein offenes 1er PO</t>
         </is>
       </c>
+      <c r="J41" t="n">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1993,6 +2116,12 @@
       <c r="H42" t="n">
         <v>0</v>
       </c>
+      <c r="I42" t="n">
+        <v/>
+      </c>
+      <c r="J42" t="n">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2025,6 +2154,9 @@
       <c r="H43" t="n">
         <v>1</v>
       </c>
+      <c r="I43" t="n">
+        <v/>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>online</t>
@@ -2062,6 +2194,9 @@
       <c r="H44" t="n">
         <v>1</v>
       </c>
+      <c r="I44" t="n">
+        <v/>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>online</t>
@@ -2099,6 +2234,9 @@
       <c r="H45" t="n">
         <v>1</v>
       </c>
+      <c r="I45" t="n">
+        <v/>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>online</t>
@@ -2136,6 +2274,9 @@
       <c r="H46" t="n">
         <v>1</v>
       </c>
+      <c r="I46" t="n">
+        <v/>
+      </c>
       <c r="J46" t="inlineStr">
         <is>
           <t>online</t>
@@ -2173,6 +2314,9 @@
       <c r="H47" t="n">
         <v>1</v>
       </c>
+      <c r="I47" t="n">
+        <v/>
+      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>online</t>
@@ -2210,6 +2354,9 @@
       <c r="H48" t="n">
         <v>1</v>
       </c>
+      <c r="I48" t="n">
+        <v/>
+      </c>
       <c r="J48" t="inlineStr">
         <is>
           <t>online</t>
@@ -2247,6 +2394,9 @@
       <c r="H49" t="n">
         <v>1</v>
       </c>
+      <c r="I49" t="n">
+        <v/>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>online</t>
@@ -2284,6 +2434,9 @@
       <c r="H50" t="n">
         <v>1</v>
       </c>
+      <c r="I50" t="n">
+        <v/>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>online</t>
@@ -2321,6 +2474,9 @@
       <c r="H51" t="n">
         <v>1</v>
       </c>
+      <c r="I51" t="n">
+        <v/>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
           <t>online</t>
@@ -2358,6 +2514,9 @@
       <c r="H52" t="n">
         <v>1</v>
       </c>
+      <c r="I52" t="n">
+        <v/>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
           <t>online</t>
@@ -2395,7 +2554,47 @@
       <c r="H53" t="n">
         <v>0</v>
       </c>
+      <c r="I53" t="n">
+        <v/>
+      </c>
       <c r="J53" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>6abdf0079d4953efea4aac6f</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Dumm, des isses!</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>10</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>46306</v>
+      </c>
+      <c r="F54" t="n">
+        <v>5</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1</v>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2412,7 +2611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6490,6 +6689,75 @@
         </is>
       </c>
       <c r="E177" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>6abdf0079d4953efea4aac6f</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>10</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>6abdf0079d4953efea4aac6f</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>2</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Hacan</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>6abdf0079d4953efea4aac6f</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>7</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Muaat</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>